<commit_message>
more various modeling improvements and bar records update
</commit_message>
<xml_diff>
--- a/data/bars.xlsx
+++ b/data/bars.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Natha\projects_and_clubs\Queen-s-Engineering-Jacket-GPA-Planner\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4206DB98-3746-4A94-9ED8-875EECDE57E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9A87C7A-EBE2-4345-8988-81931EDEB8C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{1C6F1F17-E6F1-46B7-9E88-A2681932F042}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7639" uniqueCount="1655">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7749" uniqueCount="1655">
   <si>
     <t>include</t>
   </si>
@@ -8955,7 +8955,7 @@
         <v>230</v>
       </c>
       <c r="C100" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D100" t="s">
         <v>13</v>
@@ -9060,7 +9060,7 @@
         <v>236</v>
       </c>
       <c r="C103" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D103" t="s">
         <v>13</v>
@@ -9130,7 +9130,7 @@
         <v>240</v>
       </c>
       <c r="C105" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D105" t="s">
         <v>13</v>
@@ -9165,7 +9165,7 @@
         <v>242</v>
       </c>
       <c r="C106" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D106" t="s">
         <v>13</v>
@@ -9514,9 +9514,6 @@
       <c r="B116" t="s">
         <v>265</v>
       </c>
-      <c r="C116" t="s">
-        <v>13</v>
-      </c>
       <c r="D116" t="s">
         <v>13</v>
       </c>
@@ -9725,7 +9722,7 @@
         <v>277</v>
       </c>
       <c r="C122" t="s">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="D122" t="s">
         <v>13</v>
@@ -10110,7 +10107,7 @@
         <v>301</v>
       </c>
       <c r="C133" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D133" t="s">
         <v>13</v>
@@ -10145,7 +10142,7 @@
         <v>303</v>
       </c>
       <c r="C134" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D134" t="s">
         <v>13</v>
@@ -10180,7 +10177,7 @@
         <v>305</v>
       </c>
       <c r="C135" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D135" t="s">
         <v>13</v>
@@ -10215,7 +10212,7 @@
         <v>307</v>
       </c>
       <c r="C136" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D136" t="s">
         <v>13</v>
@@ -10250,7 +10247,7 @@
         <v>309</v>
       </c>
       <c r="C137" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D137" t="s">
         <v>13</v>
@@ -10320,7 +10317,7 @@
         <v>313</v>
       </c>
       <c r="C139" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D139" t="s">
         <v>13</v>
@@ -10355,7 +10352,7 @@
         <v>315</v>
       </c>
       <c r="C140" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D140" t="s">
         <v>13</v>
@@ -10530,7 +10527,7 @@
         <v>325</v>
       </c>
       <c r="C145" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D145" t="s">
         <v>13</v>
@@ -10635,7 +10632,7 @@
         <v>331</v>
       </c>
       <c r="C148" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D148" t="s">
         <v>13</v>
@@ -10705,7 +10702,7 @@
         <v>335</v>
       </c>
       <c r="C150" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D150" t="s">
         <v>13</v>
@@ -10810,7 +10807,7 @@
         <v>341</v>
       </c>
       <c r="C153" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="D153" t="s">
         <v>13</v>
@@ -10880,7 +10877,7 @@
         <v>345</v>
       </c>
       <c r="C155" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D155" t="s">
         <v>13</v>
@@ -10950,7 +10947,7 @@
         <v>349</v>
       </c>
       <c r="C157" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D157" t="s">
         <v>13</v>
@@ -11084,13 +11081,13 @@
     </row>
     <row r="161" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A161" t="s">
-        <v>11</v>
+        <v>98</v>
       </c>
       <c r="B161" t="s">
         <v>357</v>
       </c>
       <c r="C161" t="s">
-        <v>13</v>
+        <v>100</v>
       </c>
       <c r="D161" t="s">
         <v>13</v>
@@ -11125,7 +11122,7 @@
         <v>359</v>
       </c>
       <c r="C162" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D162" t="s">
         <v>13</v>
@@ -11195,7 +11192,7 @@
         <v>363</v>
       </c>
       <c r="C164" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D164" t="s">
         <v>13</v>
@@ -11265,7 +11262,7 @@
         <v>367</v>
       </c>
       <c r="C166" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="D166" t="s">
         <v>13</v>
@@ -11300,7 +11297,7 @@
         <v>369</v>
       </c>
       <c r="C167" t="s">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="D167" t="s">
         <v>13</v>
@@ -11335,7 +11332,7 @@
         <v>371</v>
       </c>
       <c r="C168" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="D168" t="s">
         <v>13</v>
@@ -11370,7 +11367,7 @@
         <v>373</v>
       </c>
       <c r="C169" t="s">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="D169" t="s">
         <v>13</v>
@@ -11440,7 +11437,7 @@
         <v>377</v>
       </c>
       <c r="C171" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D171" t="s">
         <v>13</v>
@@ -11510,7 +11507,7 @@
         <v>382</v>
       </c>
       <c r="C173" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D173" t="s">
         <v>13</v>
@@ -11545,7 +11542,7 @@
         <v>384</v>
       </c>
       <c r="C174" t="s">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="D174" t="s">
         <v>13</v>
@@ -11580,7 +11577,7 @@
         <v>386</v>
       </c>
       <c r="C175" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D175" t="s">
         <v>13</v>
@@ -11615,7 +11612,7 @@
         <v>388</v>
       </c>
       <c r="C176" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D176" t="s">
         <v>13</v>
@@ -11650,7 +11647,7 @@
         <v>390</v>
       </c>
       <c r="C177" t="s">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="D177" t="s">
         <v>13</v>
@@ -11685,7 +11682,7 @@
         <v>392</v>
       </c>
       <c r="C178" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D178" t="s">
         <v>13</v>
@@ -11720,7 +11717,7 @@
         <v>394</v>
       </c>
       <c r="C179" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D179" t="s">
         <v>13</v>
@@ -11784,13 +11781,13 @@
     </row>
     <row r="181" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A181" t="s">
-        <v>11</v>
+        <v>98</v>
       </c>
       <c r="B181" t="s">
         <v>398</v>
       </c>
       <c r="C181" t="s">
-        <v>13</v>
+        <v>100</v>
       </c>
       <c r="D181" t="s">
         <v>13</v>
@@ -11825,7 +11822,7 @@
         <v>400</v>
       </c>
       <c r="C182" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D182" t="s">
         <v>13</v>
@@ -11860,7 +11857,7 @@
         <v>402</v>
       </c>
       <c r="C183" t="s">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="D183" t="s">
         <v>13</v>
@@ -11895,7 +11892,7 @@
         <v>404</v>
       </c>
       <c r="C184" t="s">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="D184" t="s">
         <v>13</v>
@@ -11965,7 +11962,7 @@
         <v>409</v>
       </c>
       <c r="C186" t="s">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="D186" t="s">
         <v>13</v>
@@ -12035,7 +12032,7 @@
         <v>414</v>
       </c>
       <c r="C188" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D188" t="s">
         <v>13</v>
@@ -12140,7 +12137,7 @@
         <v>421</v>
       </c>
       <c r="C191" t="s">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="D191" t="s">
         <v>13</v>
@@ -12175,7 +12172,7 @@
         <v>423</v>
       </c>
       <c r="C192" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D192" t="s">
         <v>13</v>
@@ -12245,7 +12242,7 @@
         <v>428</v>
       </c>
       <c r="C194" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D194" t="s">
         <v>13</v>
@@ -12315,7 +12312,7 @@
         <v>432</v>
       </c>
       <c r="C196" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D196" t="s">
         <v>13</v>
@@ -12350,7 +12347,7 @@
         <v>434</v>
       </c>
       <c r="C197" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D197" t="s">
         <v>13</v>
@@ -12385,7 +12382,7 @@
         <v>436</v>
       </c>
       <c r="C198" t="s">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="D198" t="s">
         <v>13</v>
@@ -12420,7 +12417,7 @@
         <v>438</v>
       </c>
       <c r="C199" t="s">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="D199" t="s">
         <v>13</v>
@@ -12490,7 +12487,7 @@
         <v>442</v>
       </c>
       <c r="C201" t="s">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="D201" t="s">
         <v>13</v>
@@ -12525,7 +12522,7 @@
         <v>444</v>
       </c>
       <c r="C202" t="s">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="D202" t="s">
         <v>13</v>
@@ -12560,7 +12557,7 @@
         <v>446</v>
       </c>
       <c r="C203" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D203" t="s">
         <v>13</v>
@@ -12595,7 +12592,7 @@
         <v>448</v>
       </c>
       <c r="C204" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D204" t="s">
         <v>13</v>
@@ -12630,7 +12627,7 @@
         <v>450</v>
       </c>
       <c r="C205" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D205" t="s">
         <v>13</v>
@@ -12665,7 +12662,7 @@
         <v>452</v>
       </c>
       <c r="C206" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D206" t="s">
         <v>13</v>
@@ -12700,7 +12697,7 @@
         <v>454</v>
       </c>
       <c r="C207" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D207" t="s">
         <v>13</v>
@@ -12805,7 +12802,7 @@
         <v>460</v>
       </c>
       <c r="C210" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="D210" t="s">
         <v>13</v>
@@ -12910,7 +12907,7 @@
         <v>466</v>
       </c>
       <c r="C213" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D213" t="s">
         <v>13</v>
@@ -12945,7 +12942,7 @@
         <v>468</v>
       </c>
       <c r="C214" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D214" t="s">
         <v>13</v>
@@ -12974,13 +12971,13 @@
     </row>
     <row r="215" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A215" t="s">
-        <v>11</v>
+        <v>98</v>
       </c>
       <c r="B215" t="s">
         <v>470</v>
       </c>
       <c r="C215" t="s">
-        <v>13</v>
+        <v>100</v>
       </c>
       <c r="D215" t="s">
         <v>13</v>
@@ -13015,7 +13012,7 @@
         <v>472</v>
       </c>
       <c r="C216" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D216" t="s">
         <v>13</v>
@@ -13050,7 +13047,7 @@
         <v>474</v>
       </c>
       <c r="C217" t="s">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="D217" t="s">
         <v>13</v>
@@ -13120,7 +13117,7 @@
         <v>478</v>
       </c>
       <c r="C219" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="D219" t="s">
         <v>13</v>
@@ -13155,7 +13152,7 @@
         <v>480</v>
       </c>
       <c r="C220" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D220" t="s">
         <v>13</v>
@@ -13190,7 +13187,7 @@
         <v>482</v>
       </c>
       <c r="C221" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D221" t="s">
         <v>13</v>
@@ -13225,7 +13222,7 @@
         <v>484</v>
       </c>
       <c r="C222" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D222" t="s">
         <v>13</v>
@@ -13400,7 +13397,7 @@
         <v>495</v>
       </c>
       <c r="C227" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D227" t="s">
         <v>13</v>
@@ -13435,7 +13432,7 @@
         <v>497</v>
       </c>
       <c r="C228" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="D228" t="s">
         <v>13</v>
@@ -13540,7 +13537,7 @@
         <v>503</v>
       </c>
       <c r="C231" t="s">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="D231" t="s">
         <v>13</v>
@@ -13575,7 +13572,7 @@
         <v>505</v>
       </c>
       <c r="C232" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="D232" t="s">
         <v>13</v>
@@ -13645,7 +13642,7 @@
         <v>508</v>
       </c>
       <c r="C234" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D234" t="s">
         <v>13</v>
@@ -13785,7 +13782,7 @@
         <v>516</v>
       </c>
       <c r="C238" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D238" t="s">
         <v>13</v>
@@ -13820,7 +13817,7 @@
         <v>518</v>
       </c>
       <c r="C239" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D239" t="s">
         <v>13</v>
@@ -13890,7 +13887,7 @@
         <v>522</v>
       </c>
       <c r="C241" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D241" t="s">
         <v>13</v>
@@ -14030,7 +14027,7 @@
         <v>530</v>
       </c>
       <c r="C245" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D245" t="s">
         <v>13</v>
@@ -14065,7 +14062,7 @@
         <v>532</v>
       </c>
       <c r="C246" t="s">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="D246" t="s">
         <v>13</v>
@@ -14100,7 +14097,7 @@
         <v>534</v>
       </c>
       <c r="C247" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="D247" t="s">
         <v>13</v>
@@ -14135,7 +14132,7 @@
         <v>536</v>
       </c>
       <c r="C248" t="s">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="D248" t="s">
         <v>13</v>
@@ -14520,7 +14517,7 @@
         <v>559</v>
       </c>
       <c r="C259" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="D259" t="s">
         <v>13</v>

</xml_diff>

<commit_message>
added quebec flag and street signs
</commit_message>
<xml_diff>
--- a/data/bars.xlsx
+++ b/data/bars.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Natha\projects_and_clubs\Queen-s-Engineering-Jacket-GPA-Planner\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF978DE5-34D5-4400-84F1-9807FD468F4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89CBF795-1508-4D57-92DE-CB30F721F433}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{1C6F1F17-E6F1-46B7-9E88-A2681932F042}"/>
   </bookViews>
@@ -6886,13 +6886,13 @@
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>98</v>
+        <v>11</v>
       </c>
       <c r="B38" t="s">
         <v>99</v>
       </c>
       <c r="C38" t="s">
-        <v>100</v>
+        <v>19</v>
       </c>
       <c r="D38" t="s">
         <v>13</v>

</xml_diff>

<commit_message>
added a tutorial button
a diagram will show up highlighted showing the users where things go
</commit_message>
<xml_diff>
--- a/data/bars.xlsx
+++ b/data/bars.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Natha\projects_and_clubs\Queen-s-Engineering-Jacket-GPA-Planner\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{944C26D7-01CC-4964-8B38-4411D6FF6379}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E96B334-0B54-4F6D-8CED-E4B30C7F0713}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{1C6F1F17-E6F1-46B7-9E88-A2681932F042}"/>
   </bookViews>
@@ -33086,7 +33086,7 @@
     </row>
     <row r="787" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A787" t="s">
-        <v>11</v>
+        <v>98</v>
       </c>
       <c r="B787" t="s">
         <v>1635</v>

</xml_diff>